<commit_message>
1st update to successfully build and setup the project in VScode
</commit_message>
<xml_diff>
--- a/src/test/resources/testdataCMS/GetProductInfo.xlsx
+++ b/src/test/resources/testdataCMS/GetProductInfo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="36">
   <si>
     <t>No</t>
   </si>
@@ -116,6 +116,18 @@
   </si>
   <si>
     <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Giỏ quà Tết attip</t>
+  </si>
+  <si>
+    <t>$5,000,000.00</t>
+  </si>
+  <si>
+    <t>16</t>
   </si>
 </sst>
 </file>
@@ -173,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -201,6 +213,36 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -597,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" style="1" width="9.0"/>
@@ -863,6 +905,40 @@
         <v>24</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="s" s="50">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s" s="51">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s" s="52">
+        <v>34</v>
+      </c>
+      <c r="D16" t="s" s="53">
+        <v>19</v>
+      </c>
+      <c r="E16" t="s" s="54">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="55">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s" s="56">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s" s="57">
+        <v>34</v>
+      </c>
+      <c r="D17" t="s" s="58">
+        <v>19</v>
+      </c>
+      <c r="E17" t="s" s="59">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Framewrok for better scalability
</commit_message>
<xml_diff>
--- a/src/test/resources/testdataCMS/GetProductInfo.xlsx
+++ b/src/test/resources/testdataCMS/GetProductInfo.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="43">
   <si>
     <t>No</t>
   </si>
@@ -128,6 +128,27 @@
   </si>
   <si>
     <t>16</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Giỏ quà Tết hQcVi</t>
   </si>
 </sst>
 </file>
@@ -185,7 +206,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -213,6 +234,96 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -639,7 +750,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" style="1" width="9.0"/>
@@ -939,6 +1050,108 @@
         <v>24</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="s" s="60">
+        <v>36</v>
+      </c>
+      <c r="B18" t="s" s="61">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s" s="62">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s" s="63">
+        <v>19</v>
+      </c>
+      <c r="E18" t="s" s="64">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="65">
+        <v>37</v>
+      </c>
+      <c r="B19" t="s" s="66">
+        <v>33</v>
+      </c>
+      <c r="C19" t="s" s="67">
+        <v>34</v>
+      </c>
+      <c r="D19" t="s" s="68">
+        <v>19</v>
+      </c>
+      <c r="E19" t="s" s="69">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="70">
+        <v>38</v>
+      </c>
+      <c r="B20" t="s" s="71">
+        <v>33</v>
+      </c>
+      <c r="C20" t="s" s="72">
+        <v>34</v>
+      </c>
+      <c r="D20" t="s" s="73">
+        <v>19</v>
+      </c>
+      <c r="E20" t="s" s="74">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="75">
+        <v>39</v>
+      </c>
+      <c r="B21" t="s" s="76">
+        <v>33</v>
+      </c>
+      <c r="C21" t="s" s="77">
+        <v>34</v>
+      </c>
+      <c r="D21" t="s" s="78">
+        <v>19</v>
+      </c>
+      <c r="E21" t="s" s="79">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="80">
+        <v>40</v>
+      </c>
+      <c r="B22" t="s" s="81">
+        <v>33</v>
+      </c>
+      <c r="C22" t="s" s="82">
+        <v>34</v>
+      </c>
+      <c r="D22" t="s" s="83">
+        <v>19</v>
+      </c>
+      <c r="E22" t="s" s="84">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="85">
+        <v>41</v>
+      </c>
+      <c r="B23" t="s" s="86">
+        <v>42</v>
+      </c>
+      <c r="C23" t="s" s="87">
+        <v>34</v>
+      </c>
+      <c r="D23" t="s" s="88">
+        <v>19</v>
+      </c>
+      <c r="E23" t="s" s="89">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>